<commit_message>
Update dashboard/data (2026-07-23 10:40)
</commit_message>
<xml_diff>
--- a/Defect_Report.xlsx
+++ b/Defect_Report.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44F13FE1-B81D-4425-A305-6F7F2D16DFFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{44F13FE1-B81D-4425-A305-6F7F2D16DFFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8B379D7-100A-41E9-8B50-E94C6C693C56}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04FC0AC7-FBBE-4BBC-BC06-125512EACFB3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
   <si>
     <t>วันที่ / Date</t>
   </si>
@@ -78,6 +78,60 @@
   </si>
   <si>
     <t>รูป หลังแก้</t>
+  </si>
+  <si>
+    <t>PhanasonSamutprakhan Residence</t>
+  </si>
+  <si>
+    <t>1ERV-01</t>
+  </si>
+  <si>
+    <t>ปริมาณลมในแบบผู้รับเหมาทำมาไม่ตรงกับรูปอ้างอิง</t>
+  </si>
+  <si>
+    <t>สูง / High</t>
+  </si>
+  <si>
+    <t>กำลังแก้ / In Progress</t>
+  </si>
+  <si>
+    <t>3T</t>
+  </si>
+  <si>
+    <t>S’rin House</t>
+  </si>
+  <si>
+    <t>ห้องกล๊ออฟ</t>
+  </si>
+  <si>
+    <t>รองานโครงสร้าง</t>
+  </si>
+  <si>
+    <t>ต่ำ / Low</t>
+  </si>
+  <si>
+    <t>เปิด / รอ</t>
+  </si>
+  <si>
+    <t>บริษัท เคบีเอส ซีสเต็ม จํากัด</t>
+  </si>
+  <si>
+    <t>รอวันที่สามารถเข้าทำงานได้</t>
+  </si>
+  <si>
+    <t>HUAY KWANG RESIDENCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">รอสรุปหลัง Site meeting </t>
+  </si>
+  <si>
+    <t>Site meeting ก่อนเริ่มงาน 7/24/2026</t>
+  </si>
+  <si>
+    <t>บ้านคุณเต้ย</t>
+  </si>
+  <si>
+    <t>เริ่มงานได้ 3 สิงหา</t>
   </si>
 </sst>
 </file>
@@ -542,7 +596,8 @@
   <dimension ref="A1:M53"/>
   <sheetFormatPr defaultRowHeight="16.8" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="2" width="14.77734375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="40.77734375" style="1" customWidth="1"/>
     <col min="5" max="5" width="16.77734375" style="1" customWidth="1"/>
@@ -641,57 +696,113 @@
       <c r="M4" s="7"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="A5" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="2">
+        <v>46227</v>
+      </c>
+      <c r="I5" s="2">
+        <v>46227</v>
+      </c>
       <c r="J5" s="4"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
       <c r="M5" s="7"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="A6" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
-      <c r="J6" s="4"/>
+      <c r="J6" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="7"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
+      <c r="A7" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="D7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="G7" s="3"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
-      <c r="J7" s="4"/>
+      <c r="J7" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
       <c r="M7" s="7"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
+      <c r="A8" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="C8" s="3"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+      <c r="D8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="G8" s="3"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -1379,12 +1490,18 @@
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E39" xr:uid="{1D76DD1E-3D77-457B-B34F-44BCC2B367B7}">
       <formula1>"ต่ำ / Low,ปานกลาง / Medium,สูง / High,วิกฤต / Critical"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F39" xr:uid="{9142C414-FBEE-4106-981C-B95747E09F3E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F5 F21:F39" xr:uid="{9142C414-FBEE-4106-981C-B95747E09F3E}">
       <formula1>"เปิด / Open,กำลังแก้ / In Progress,แก้เสร็จ / Fixed,ปิด / Closed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F13:F20" xr:uid="{CDB5D18A-3777-490D-9FBC-6359E5CBE300}">
+      <formula1>"เปิด / รอ,กำลังแก้ / In Progress,แก้เสร็จ / Fixed,ปิด / Closed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6:F12" xr:uid="{60ECFCFC-3AD4-4842-BAB6-A7EB051C8426}">
+      <formula1>"Wait/ รอ,กำลังแก้ / In Progress,แก้เสร็จ / Fixed,ปิด / Closed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1393,6 +1510,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -1645,15 +1771,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1668,13 +1785,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23449C61-D5BA-44B1-A472-FB4C9EEC61EE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF18A786-B973-49B0-99B2-5E7AF5814A3A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF18A786-B973-49B0-99B2-5E7AF5814A3A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23449C61-D5BA-44B1-A472-FB4C9EEC61EE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9B76825-6942-4800-BFAC-87DF8A7A9F61}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9B76825-6942-4800-BFAC-87DF8A7A9F61}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 11:00)
</commit_message>
<xml_diff>
--- a/Defect_Report.xlsx
+++ b/Defect_Report.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Report/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{44F13FE1-B81D-4425-A305-6F7F2D16DFFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8B379D7-100A-41E9-8B50-E94C6C693C56}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FD5B063-C227-4A0F-8154-A968E17D40D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04FC0AC7-FBBE-4BBC-BC06-125512EACFB3}"/>
   </bookViews>
@@ -38,8 +38,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="43">
   <si>
     <t>วันที่ / Date</t>
   </si>
@@ -110,9 +132,6 @@
     <t>ต่ำ / Low</t>
   </si>
   <si>
-    <t>เปิด / รอ</t>
-  </si>
-  <si>
     <t>บริษัท เคบีเอส ซีสเต็ม จํากัด</t>
   </si>
   <si>
@@ -132,6 +151,45 @@
   </si>
   <si>
     <t>เริ่มงานได้ 3 สิงหา</t>
+  </si>
+  <si>
+    <t>Wait/ รอ</t>
+  </si>
+  <si>
+    <t>บริษัท อาร์ทอพ แอร์ ซัพพลาย จำกัด</t>
+  </si>
+  <si>
+    <t>นายคธาชัย จันทร์ศรี</t>
+  </si>
+  <si>
+    <t>หมู่บ้านมัณฑนา</t>
+  </si>
+  <si>
+    <t>รองานโครงสร้าง ปลายเดือน 7</t>
+  </si>
+  <si>
+    <t>บริษัทเอ.เอ็น.เอ็นจิเนียริ่งจํากัด</t>
+  </si>
+  <si>
+    <t>บ้านคุณปุกกี้</t>
+  </si>
+  <si>
+    <t>เริ่มงานได้เดือน 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">บ้านบางบอน5ซอย7 </t>
+  </si>
+  <si>
+    <t>เดือน 8 ติดตามสถานะ โปรเจค</t>
+  </si>
+  <si>
+    <t>Main Con กำลังแก้แนวท่อไฟ</t>
+  </si>
+  <si>
+    <t>คุณทวีชัย สมุทรปราการ</t>
+  </si>
+  <si>
+    <t>รองานโครงสร้าง / Site Meeting 8/04/2026</t>
   </si>
 </sst>
 </file>
@@ -274,6 +332,70 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -602,10 +724,11 @@
     <col min="4" max="4" width="40.77734375" style="1" customWidth="1"/>
     <col min="5" max="5" width="16.77734375" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="18.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="14.77734375" style="1" customWidth="1"/>
     <col min="10" max="10" width="25.77734375" style="1" customWidth="1"/>
-    <col min="11" max="12" width="20.77734375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="34.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="20.77734375" style="1" customWidth="1"/>
     <col min="13" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
@@ -695,7 +818,7 @@
       <c r="L4" s="3"/>
       <c r="M4" s="7"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:13" ht="107.4" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="2">
         <v>46226</v>
       </c>
@@ -724,7 +847,9 @@
         <v>46227</v>
       </c>
       <c r="J5" s="4"/>
-      <c r="K5" s="3"/>
+      <c r="K5" s="3" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="L5" s="3"/>
       <c r="M5" s="7"/>
     </row>
@@ -745,15 +870,15 @@
         <v>22</v>
       </c>
       <c r="F6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
@@ -764,23 +889,25 @@
         <v>46226</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G7" s="3"/>
+        <v>30</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>31</v>
+      </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
@@ -791,35 +918,53 @@
         <v>46226</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G8" s="3"/>
+        <v>30</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
-      <c r="J8" s="4"/>
+      <c r="J8" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
       <c r="M8" s="7"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
+      <c r="A9" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="2"/>
+      <c r="D9" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="2">
+        <v>46233</v>
+      </c>
       <c r="I9" s="2"/>
       <c r="J9" s="4"/>
       <c r="K9" s="3"/>
@@ -827,14 +972,26 @@
       <c r="M9" s="7"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
+      <c r="A10" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="C10" s="3"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
+      <c r="D10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="G10" s="3"/>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2">
+        <v>46264</v>
+      </c>
       <c r="I10" s="2"/>
       <c r="J10" s="4"/>
       <c r="K10" s="3"/>
@@ -842,14 +999,28 @@
       <c r="M10" s="7"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
+      <c r="A11" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>38</v>
+      </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="2"/>
+      <c r="D11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="2">
+        <v>46249</v>
+      </c>
       <c r="I11" s="2"/>
       <c r="J11" s="4"/>
       <c r="K11" s="3"/>
@@ -857,13 +1028,25 @@
       <c r="M11" s="7"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
+      <c r="A12" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
+      <c r="D12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="4"/>
@@ -1510,15 +1693,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -1771,6 +1945,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1785,14 +1968,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF18A786-B973-49B0-99B2-5E7AF5814A3A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23449C61-D5BA-44B1-A472-FB4C9EEC61EE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1811,6 +1986,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF18A786-B973-49B0-99B2-5E7AF5814A3A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9B76825-6942-4800-BFAC-87DF8A7A9F61}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 11:50)
</commit_message>
<xml_diff>
--- a/Defect_Report.xlsx
+++ b/Defect_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FD5B063-C227-4A0F-8154-A968E17D40D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292D2A6E-DC0D-4DB6-8E62-8ACE19513C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04FC0AC7-FBBE-4BBC-BC06-125512EACFB3}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
   <si>
     <t>วันที่ / Date</t>
   </si>
@@ -165,9 +165,6 @@
     <t>หมู่บ้านมัณฑนา</t>
   </si>
   <si>
-    <t>รองานโครงสร้าง ปลายเดือน 7</t>
-  </si>
-  <si>
     <t>บริษัทเอ.เอ็น.เอ็นจิเนียริ่งจํากัด</t>
   </si>
   <si>
@@ -190,6 +187,18 @@
   </si>
   <si>
     <t>รองานโครงสร้าง / Site Meeting 8/04/2026</t>
+  </si>
+  <si>
+    <t>Sukhumvit 77 Prawet Residence</t>
+  </si>
+  <si>
+    <t>รอส่งมอบงาน</t>
+  </si>
+  <si>
+    <t>ปานกลาง / Medium</t>
+  </si>
+  <si>
+    <t>กำลังขึ้นส่วนของหลังคาขั้น 2  ยังไม่สามารถเข้าทำงานได้</t>
   </si>
 </sst>
 </file>
@@ -841,7 +850,7 @@
         <v>18</v>
       </c>
       <c r="H5" s="2">
-        <v>46227</v>
+        <v>46226</v>
       </c>
       <c r="I5" s="2">
         <v>46227</v>
@@ -936,7 +945,7 @@
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
@@ -951,7 +960,7 @@
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="4" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>22</v>
@@ -960,7 +969,7 @@
         <v>30</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H9" s="2">
         <v>46233</v>
@@ -976,11 +985,11 @@
         <v>46226</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>22</v>
@@ -1003,11 +1012,11 @@
         <v>46226</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>22</v>
@@ -1016,7 +1025,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H11" s="2">
         <v>46249</v>
@@ -1032,11 +1041,11 @@
         <v>46226</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>22</v>
@@ -1055,14 +1064,28 @@
       <c r="M12" s="7"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="A13" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="2"/>
+      <c r="D13" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H13" s="2">
+        <v>46239</v>
+      </c>
       <c r="I13" s="2"/>
       <c r="J13" s="4"/>
       <c r="K13" s="3"/>
@@ -1680,10 +1703,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F5 F21:F39" xr:uid="{9142C414-FBEE-4106-981C-B95747E09F3E}">
       <formula1>"เปิด / Open,กำลังแก้ / In Progress,แก้เสร็จ / Fixed,ปิด / Closed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F13:F20" xr:uid="{CDB5D18A-3777-490D-9FBC-6359E5CBE300}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F14:F20" xr:uid="{CDB5D18A-3777-490D-9FBC-6359E5CBE300}">
       <formula1>"เปิด / รอ,กำลังแก้ / In Progress,แก้เสร็จ / Fixed,ปิด / Closed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6:F12" xr:uid="{60ECFCFC-3AD4-4842-BAB6-A7EB051C8426}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6:F13" xr:uid="{60ECFCFC-3AD4-4842-BAB6-A7EB051C8426}">
       <formula1>"Wait/ รอ,กำลังแก้ / In Progress,แก้เสร็จ / Fixed,ปิด / Closed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1946,15 +1969,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
@@ -1965,6 +1979,15 @@
     <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1987,14 +2010,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF18A786-B973-49B0-99B2-5E7AF5814A3A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9B76825-6942-4800-BFAC-87DF8A7A9F61}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2003,4 +2018,12 @@
     <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF18A786-B973-49B0-99B2-5E7AF5814A3A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 11:56)
</commit_message>
<xml_diff>
--- a/Defect_Report.xlsx
+++ b/Defect_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292D2A6E-DC0D-4DB6-8E62-8ACE19513C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F02B2AC-815D-42F3-A0FD-6095082C3EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04FC0AC7-FBBE-4BBC-BC06-125512EACFB3}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="46">
   <si>
     <t>วันที่ / Date</t>
   </si>
@@ -997,7 +997,9 @@
       <c r="F10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="G10" s="3"/>
+      <c r="G10" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="H10" s="2">
         <v>46264</v>
       </c>

</xml_diff>

<commit_message>
Update dashboard/data (2026-07-23 12:07)
</commit_message>
<xml_diff>
--- a/Defect_Report.xlsx
+++ b/Defect_Report.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\OneDrive - Coral Life\Coral Life - BA - Solution Design 1\1_Non-Project\7_Engineer\IAQ Solution\0_ERV Management\2_Construction Management\Report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corallife806.sharepoint.com/sites/CoralLife2/Document Sharing/BA - Solution Design/1_Non-Project/7_Engineer/IAQ Solution/0_ERV Management/2_Construction Management/Report/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F02B2AC-815D-42F3-A0FD-6095082C3EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -1718,6 +1718,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
+    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008ED2D49705E83042817996DE5E733B41" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba94834c452bdfc5c8776e4d6f86dfb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xmlns:ns3="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ff4bedaaabc80ab55b5467b16ce003eb" ns2:_="" ns3:_="">
     <xsd:import namespace="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
@@ -1970,29 +1992,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Complete xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d1b07a1-7849-4740-a4b1-3343cd5aadb6" xsi:nil="true"/>
-    <DateStart xmlns="d1b9d38e-82c4-40dd-a627-c28ab9108e1c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF18A786-B973-49B0-99B2-5E7AF5814A3A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9B76825-6942-4800-BFAC-87DF8A7A9F61}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
+    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23449C61-D5BA-44B1-A472-FB4C9EEC61EE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2009,23 +2028,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9B76825-6942-4800-BFAC-87DF8A7A9F61}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d1b9d38e-82c4-40dd-a627-c28ab9108e1c"/>
-    <ds:schemaRef ds:uri="2d1b07a1-7849-4740-a4b1-3343cd5aadb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF18A786-B973-49B0-99B2-5E7AF5814A3A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>